<commit_message>
Hardcode Household Revenue income figures for the clinical demo scenario
D21 (Applicant Primary / Wages-Salary): \$400 Weekly -> \$25,500 Annual
D22 (Spouse/Other / Part-Time): \$100 Weekly -> \$5,200 Annual

These were the original uploaded template's placeholder sample values --
replaced with the demo scenario's real figures directly in the template
itself (rather than in fqhcExport.js), since nothing in the FQHC Intake
form reports household income, so these are fixed for every export, the
same way Mary/Sam/Tina's household details are. Existing currency
formatting and the annualization formulas (F21/F22/F24) are untouched --
Excel recalculates those automatically on open.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lv2brQXZjSF8iUMTHu3qfQ
</commit_message>
<xml_diff>
--- a/dde-webhook/assets/fqhc-sliding-fee-scale-template.xlsx
+++ b/dde-webhook/assets/fqhc-sliding-fee-scale-template.xlsx
@@ -872,11 +872,11 @@
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>400</v>
+        <v>25500</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Weekly</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="F21" s="12">
@@ -896,11 +896,11 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>100</v>
+        <v>5200</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Weekly</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="F22" s="12">

</xml_diff>